<commit_message>
Definitiestudie leeuwarden app en trailerhellingen
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Mathijs.xlsx
+++ b/Logboeken/Logboek Mathijs.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>Datum</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>Uitwerken planning</t>
+  </si>
+  <si>
+    <t>Definitiestudie trailerhellingen en leeuwarden app gemaakt</t>
+  </si>
+  <si>
+    <t>3 uur</t>
   </si>
 </sst>
 </file>
@@ -118,10 +124,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -468,8 +474,8 @@
     <col min="3" max="3" width="13.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="6" customFormat="1" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:3" s="7" customFormat="1" ht="46.5" x14ac:dyDescent="0.7">
+      <c r="A1" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -477,7 +483,7 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -564,10 +570,20 @@
       <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="1"/>
+      <c r="A12" s="3">
+        <v>41024</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>

</xml_diff>

<commit_message>
Logboek update .... goh
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Mathijs.xlsx
+++ b/Logboeken/Logboek Mathijs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="11760" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="60" windowWidth="20730" windowHeight="11700" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
   <si>
     <t>Datum</t>
   </si>
@@ -166,6 +166,15 @@
   </si>
   <si>
     <t>Hoop niet opgegeven, opnieuw geprobeerd het knopje te fixen dit keer met succes!</t>
+  </si>
+  <si>
+    <t>Verder met het tweaken van de App, detailPagina verder linken aan een annotation</t>
+  </si>
+  <si>
+    <t>Omzetten van het oude project naar het nieuwe met de nieuwe structuur en opmaak (settingsWindow gedaan)</t>
+  </si>
+  <si>
+    <t>Gestoeit met een blob, wou niet morgen maar weer verder kijken</t>
   </si>
 </sst>
 </file>
@@ -574,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C315"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.125" style="1" customWidth="1"/>
@@ -1061,47 +1070,1117 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="4"/>
-      <c r="B45" s="1"/>
+      <c r="A45" s="3">
+        <v>41045</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C45" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
+      <c r="A46" s="3">
+        <v>41050</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4"/>
+      <c r="A47" s="3">
+        <v>41050</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
-      <c r="B52" s="4"/>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B78" s="1"/>
+      <c r="C78" s="1"/>
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B79" s="1"/>
+      <c r="C79" s="1"/>
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B80" s="1"/>
+      <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B81" s="1"/>
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B82" s="1"/>
+      <c r="C82" s="1"/>
+    </row>
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B84" s="1"/>
+      <c r="C84" s="1"/>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+    </row>
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+    </row>
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B89" s="1"/>
+      <c r="C89" s="1"/>
+    </row>
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B90" s="1"/>
+      <c r="C90" s="1"/>
+    </row>
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+    </row>
+    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+    </row>
+    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+    </row>
+    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+    </row>
+    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+    </row>
+    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+    </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B98" s="1"/>
+      <c r="C98" s="1"/>
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+    </row>
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+    </row>
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+    </row>
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B103" s="1"/>
+      <c r="C103" s="1"/>
+    </row>
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+    </row>
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B105" s="1"/>
+      <c r="C105" s="1"/>
+    </row>
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+    </row>
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B107" s="1"/>
+      <c r="C107" s="1"/>
+    </row>
+    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B108" s="1"/>
+      <c r="C108" s="1"/>
+    </row>
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B109" s="1"/>
+      <c r="C109" s="1"/>
+    </row>
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B110" s="1"/>
+      <c r="C110" s="1"/>
+    </row>
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B111" s="1"/>
+      <c r="C111" s="1"/>
+    </row>
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B112" s="1"/>
+      <c r="C112" s="1"/>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B113" s="1"/>
+      <c r="C113" s="1"/>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B115" s="1"/>
+      <c r="C115" s="1"/>
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B116" s="1"/>
+      <c r="C116" s="1"/>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B117" s="1"/>
+      <c r="C117" s="1"/>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B118" s="1"/>
+      <c r="C118" s="1"/>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B120" s="1"/>
+      <c r="C120" s="1"/>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B121" s="1"/>
+      <c r="C121" s="1"/>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B123" s="1"/>
+      <c r="C123" s="1"/>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B124" s="1"/>
+      <c r="C124" s="1"/>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B125" s="1"/>
+      <c r="C125" s="1"/>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B126" s="1"/>
+      <c r="C126" s="1"/>
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B127" s="1"/>
+      <c r="C127" s="1"/>
+    </row>
+    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B128" s="1"/>
+      <c r="C128" s="1"/>
+    </row>
+    <row r="129" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B129" s="1"/>
+      <c r="C129" s="1"/>
+    </row>
+    <row r="130" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B130" s="1"/>
+      <c r="C130" s="1"/>
+    </row>
+    <row r="131" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B131" s="1"/>
+      <c r="C131" s="1"/>
+    </row>
+    <row r="132" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B132" s="1"/>
+      <c r="C132" s="1"/>
+    </row>
+    <row r="133" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B133" s="1"/>
+      <c r="C133" s="1"/>
+    </row>
+    <row r="134" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B134" s="1"/>
+      <c r="C134" s="1"/>
+    </row>
+    <row r="135" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B135" s="1"/>
+      <c r="C135" s="1"/>
+    </row>
+    <row r="136" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B136" s="1"/>
+      <c r="C136" s="1"/>
+    </row>
+    <row r="137" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B137" s="1"/>
+      <c r="C137" s="1"/>
+    </row>
+    <row r="138" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B138" s="1"/>
+      <c r="C138" s="1"/>
+    </row>
+    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B139" s="1"/>
+      <c r="C139" s="1"/>
+    </row>
+    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B140" s="1"/>
+      <c r="C140" s="1"/>
+    </row>
+    <row r="141" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B141" s="1"/>
+      <c r="C141" s="1"/>
+    </row>
+    <row r="142" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B142" s="1"/>
+      <c r="C142" s="1"/>
+    </row>
+    <row r="143" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B143" s="1"/>
+      <c r="C143" s="1"/>
+    </row>
+    <row r="144" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B144" s="1"/>
+      <c r="C144" s="1"/>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B145" s="1"/>
+      <c r="C145" s="1"/>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B146" s="1"/>
+      <c r="C146" s="1"/>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B147" s="1"/>
+      <c r="C147" s="1"/>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B148" s="1"/>
+      <c r="C148" s="1"/>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B149" s="1"/>
+      <c r="C149" s="1"/>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B150" s="1"/>
+      <c r="C150" s="1"/>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B151" s="1"/>
+      <c r="C151" s="1"/>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B152" s="1"/>
+      <c r="C152" s="1"/>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B153" s="1"/>
+      <c r="C153" s="1"/>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B154" s="1"/>
+      <c r="C154" s="1"/>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B155" s="1"/>
+      <c r="C155" s="1"/>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B156" s="1"/>
+      <c r="C156" s="1"/>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B157" s="1"/>
+      <c r="C157" s="1"/>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B158" s="1"/>
+      <c r="C158" s="1"/>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B159" s="1"/>
+      <c r="C159" s="1"/>
+    </row>
+    <row r="160" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B160" s="1"/>
+      <c r="C160" s="1"/>
+    </row>
+    <row r="161" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B161" s="1"/>
+      <c r="C161" s="1"/>
+    </row>
+    <row r="162" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B162" s="1"/>
+      <c r="C162" s="1"/>
+    </row>
+    <row r="163" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B163" s="1"/>
+      <c r="C163" s="1"/>
+    </row>
+    <row r="164" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B164" s="1"/>
+      <c r="C164" s="1"/>
+    </row>
+    <row r="165" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B165" s="1"/>
+      <c r="C165" s="1"/>
+    </row>
+    <row r="166" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B166" s="1"/>
+      <c r="C166" s="1"/>
+    </row>
+    <row r="167" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B167" s="1"/>
+      <c r="C167" s="1"/>
+    </row>
+    <row r="168" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B168" s="1"/>
+      <c r="C168" s="1"/>
+    </row>
+    <row r="169" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B169" s="1"/>
+      <c r="C169" s="1"/>
+    </row>
+    <row r="170" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B170" s="1"/>
+      <c r="C170" s="1"/>
+    </row>
+    <row r="171" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B171" s="1"/>
+      <c r="C171" s="1"/>
+    </row>
+    <row r="172" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B172" s="1"/>
+      <c r="C172" s="1"/>
+    </row>
+    <row r="173" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B173" s="1"/>
+      <c r="C173" s="1"/>
+    </row>
+    <row r="174" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B174" s="1"/>
+      <c r="C174" s="1"/>
+    </row>
+    <row r="175" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B175" s="1"/>
+      <c r="C175" s="1"/>
+    </row>
+    <row r="176" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B176" s="1"/>
+      <c r="C176" s="1"/>
+    </row>
+    <row r="177" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B177" s="1"/>
+      <c r="C177" s="1"/>
+    </row>
+    <row r="178" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B178" s="1"/>
+      <c r="C178" s="1"/>
+    </row>
+    <row r="179" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B179" s="1"/>
+      <c r="C179" s="1"/>
+    </row>
+    <row r="180" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B180" s="1"/>
+      <c r="C180" s="1"/>
+    </row>
+    <row r="181" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B181" s="1"/>
+      <c r="C181" s="1"/>
+    </row>
+    <row r="182" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B182" s="1"/>
+      <c r="C182" s="1"/>
+    </row>
+    <row r="183" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B183" s="1"/>
+      <c r="C183" s="1"/>
+    </row>
+    <row r="184" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B184" s="1"/>
+      <c r="C184" s="1"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="1"/>
+      <c r="C185" s="1"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="1"/>
+      <c r="C186" s="1"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="1"/>
+      <c r="C187" s="1"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="1"/>
+      <c r="C188" s="1"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="1"/>
+      <c r="C189" s="1"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="1"/>
+      <c r="C190" s="1"/>
+    </row>
+    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B191" s="1"/>
+      <c r="C191" s="1"/>
+    </row>
+    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B192" s="1"/>
+      <c r="C192" s="1"/>
+    </row>
+    <row r="193" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B193" s="1"/>
+      <c r="C193" s="1"/>
+    </row>
+    <row r="194" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B194" s="1"/>
+      <c r="C194" s="1"/>
+    </row>
+    <row r="195" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B195" s="1"/>
+      <c r="C195" s="1"/>
+    </row>
+    <row r="196" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B196" s="1"/>
+      <c r="C196" s="1"/>
+    </row>
+    <row r="197" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B197" s="1"/>
+      <c r="C197" s="1"/>
+    </row>
+    <row r="198" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B198" s="1"/>
+      <c r="C198" s="1"/>
+    </row>
+    <row r="199" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B199" s="1"/>
+      <c r="C199" s="1"/>
+    </row>
+    <row r="200" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B200" s="1"/>
+      <c r="C200" s="1"/>
+    </row>
+    <row r="201" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B201" s="1"/>
+      <c r="C201" s="1"/>
+    </row>
+    <row r="202" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B202" s="1"/>
+      <c r="C202" s="1"/>
+    </row>
+    <row r="203" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B203" s="1"/>
+      <c r="C203" s="1"/>
+    </row>
+    <row r="204" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B204" s="1"/>
+      <c r="C204" s="1"/>
+    </row>
+    <row r="205" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B205" s="1"/>
+      <c r="C205" s="1"/>
+    </row>
+    <row r="206" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B206" s="1"/>
+      <c r="C206" s="1"/>
+    </row>
+    <row r="207" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B207" s="1"/>
+      <c r="C207" s="1"/>
+    </row>
+    <row r="208" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B208" s="1"/>
+      <c r="C208" s="1"/>
+    </row>
+    <row r="209" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B209" s="1"/>
+      <c r="C209" s="1"/>
+    </row>
+    <row r="210" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B210" s="1"/>
+      <c r="C210" s="1"/>
+    </row>
+    <row r="211" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B211" s="1"/>
+      <c r="C211" s="1"/>
+    </row>
+    <row r="212" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B212" s="1"/>
+      <c r="C212" s="1"/>
+    </row>
+    <row r="213" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B213" s="1"/>
+      <c r="C213" s="1"/>
+    </row>
+    <row r="214" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B214" s="1"/>
+      <c r="C214" s="1"/>
+    </row>
+    <row r="215" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B215" s="1"/>
+      <c r="C215" s="1"/>
+    </row>
+    <row r="216" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B216" s="1"/>
+      <c r="C216" s="1"/>
+    </row>
+    <row r="217" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B217" s="1"/>
+      <c r="C217" s="1"/>
+    </row>
+    <row r="218" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B218" s="1"/>
+      <c r="C218" s="1"/>
+    </row>
+    <row r="219" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B219" s="1"/>
+      <c r="C219" s="1"/>
+    </row>
+    <row r="220" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B220" s="1"/>
+      <c r="C220" s="1"/>
+    </row>
+    <row r="221" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B221" s="1"/>
+      <c r="C221" s="1"/>
+    </row>
+    <row r="222" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B222" s="1"/>
+      <c r="C222" s="1"/>
+    </row>
+    <row r="223" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B223" s="1"/>
+      <c r="C223" s="1"/>
+    </row>
+    <row r="224" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B224" s="1"/>
+      <c r="C224" s="1"/>
+    </row>
+    <row r="225" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B225" s="1"/>
+      <c r="C225" s="1"/>
+    </row>
+    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B226" s="1"/>
+      <c r="C226" s="1"/>
+    </row>
+    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B227" s="1"/>
+      <c r="C227" s="1"/>
+    </row>
+    <row r="228" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B228" s="1"/>
+      <c r="C228" s="1"/>
+    </row>
+    <row r="229" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B229" s="1"/>
+      <c r="C229" s="1"/>
+    </row>
+    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B230" s="1"/>
+      <c r="C230" s="1"/>
+    </row>
+    <row r="231" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B231" s="1"/>
+      <c r="C231" s="1"/>
+    </row>
+    <row r="232" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B232" s="1"/>
+      <c r="C232" s="1"/>
+    </row>
+    <row r="233" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B233" s="1"/>
+      <c r="C233" s="1"/>
+    </row>
+    <row r="234" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B234" s="1"/>
+      <c r="C234" s="1"/>
+    </row>
+    <row r="235" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B235" s="1"/>
+      <c r="C235" s="1"/>
+    </row>
+    <row r="236" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B236" s="1"/>
+      <c r="C236" s="1"/>
+    </row>
+    <row r="237" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B237" s="1"/>
+      <c r="C237" s="1"/>
+    </row>
+    <row r="238" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B238" s="1"/>
+      <c r="C238" s="1"/>
+    </row>
+    <row r="239" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B239" s="1"/>
+      <c r="C239" s="1"/>
+    </row>
+    <row r="240" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B240" s="1"/>
+      <c r="C240" s="1"/>
+    </row>
+    <row r="241" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B241" s="1"/>
+      <c r="C241" s="1"/>
+    </row>
+    <row r="242" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B242" s="1"/>
+      <c r="C242" s="1"/>
+    </row>
+    <row r="243" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B243" s="1"/>
+      <c r="C243" s="1"/>
+    </row>
+    <row r="244" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B244" s="1"/>
+      <c r="C244" s="1"/>
+    </row>
+    <row r="245" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B245" s="1"/>
+      <c r="C245" s="1"/>
+    </row>
+    <row r="246" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B246" s="1"/>
+      <c r="C246" s="1"/>
+    </row>
+    <row r="247" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B247" s="1"/>
+      <c r="C247" s="1"/>
+    </row>
+    <row r="248" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B248" s="1"/>
+      <c r="C248" s="1"/>
+    </row>
+    <row r="249" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B249" s="1"/>
+      <c r="C249" s="1"/>
+    </row>
+    <row r="250" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B250" s="1"/>
+      <c r="C250" s="1"/>
+    </row>
+    <row r="251" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B251" s="1"/>
+      <c r="C251" s="1"/>
+    </row>
+    <row r="252" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B252" s="1"/>
+      <c r="C252" s="1"/>
+    </row>
+    <row r="253" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B253" s="1"/>
+      <c r="C253" s="1"/>
+    </row>
+    <row r="254" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B254" s="1"/>
+      <c r="C254" s="1"/>
+    </row>
+    <row r="255" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B255" s="1"/>
+      <c r="C255" s="1"/>
+    </row>
+    <row r="256" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B256" s="1"/>
+      <c r="C256" s="1"/>
+    </row>
+    <row r="257" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B257" s="1"/>
+      <c r="C257" s="1"/>
+    </row>
+    <row r="258" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B258" s="1"/>
+      <c r="C258" s="1"/>
+    </row>
+    <row r="259" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B259" s="1"/>
+      <c r="C259" s="1"/>
+    </row>
+    <row r="260" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B260" s="1"/>
+      <c r="C260" s="1"/>
+    </row>
+    <row r="261" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B261" s="1"/>
+      <c r="C261" s="1"/>
+    </row>
+    <row r="262" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B262" s="1"/>
+      <c r="C262" s="1"/>
+    </row>
+    <row r="263" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B263" s="1"/>
+      <c r="C263" s="1"/>
+    </row>
+    <row r="264" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B264" s="1"/>
+      <c r="C264" s="1"/>
+    </row>
+    <row r="265" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B265" s="1"/>
+      <c r="C265" s="1"/>
+    </row>
+    <row r="266" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B266" s="1"/>
+      <c r="C266" s="1"/>
+    </row>
+    <row r="267" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B267" s="1"/>
+      <c r="C267" s="1"/>
+    </row>
+    <row r="268" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B268" s="1"/>
+      <c r="C268" s="1"/>
+    </row>
+    <row r="269" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B269" s="1"/>
+      <c r="C269" s="1"/>
+    </row>
+    <row r="270" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B270" s="1"/>
+      <c r="C270" s="1"/>
+    </row>
+    <row r="271" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B271" s="1"/>
+      <c r="C271" s="1"/>
+    </row>
+    <row r="272" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B272" s="1"/>
+      <c r="C272" s="1"/>
+    </row>
+    <row r="273" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B273" s="1"/>
+      <c r="C273" s="1"/>
+    </row>
+    <row r="274" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B274" s="1"/>
+      <c r="C274" s="1"/>
+    </row>
+    <row r="275" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B275" s="1"/>
+      <c r="C275" s="1"/>
+    </row>
+    <row r="276" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B276" s="1"/>
+      <c r="C276" s="1"/>
+    </row>
+    <row r="277" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B277" s="1"/>
+      <c r="C277" s="1"/>
+    </row>
+    <row r="278" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B278" s="1"/>
+      <c r="C278" s="1"/>
+    </row>
+    <row r="279" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B279" s="1"/>
+      <c r="C279" s="1"/>
+    </row>
+    <row r="280" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B280" s="1"/>
+      <c r="C280" s="1"/>
+    </row>
+    <row r="281" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B281" s="1"/>
+      <c r="C281" s="1"/>
+    </row>
+    <row r="282" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B282" s="1"/>
+      <c r="C282" s="1"/>
+    </row>
+    <row r="283" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B283" s="1"/>
+      <c r="C283" s="1"/>
+    </row>
+    <row r="284" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B284" s="1"/>
+      <c r="C284" s="1"/>
+    </row>
+    <row r="285" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B285" s="1"/>
+      <c r="C285" s="1"/>
+    </row>
+    <row r="286" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B286" s="1"/>
+      <c r="C286" s="1"/>
+    </row>
+    <row r="287" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B287" s="1"/>
+      <c r="C287" s="1"/>
+    </row>
+    <row r="288" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B288" s="1"/>
+      <c r="C288" s="1"/>
+    </row>
+    <row r="289" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B289" s="1"/>
+      <c r="C289" s="1"/>
+    </row>
+    <row r="290" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B290" s="1"/>
+      <c r="C290" s="1"/>
+    </row>
+    <row r="291" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B291" s="1"/>
+      <c r="C291" s="1"/>
+    </row>
+    <row r="292" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B292" s="1"/>
+      <c r="C292" s="1"/>
+    </row>
+    <row r="293" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B293" s="1"/>
+      <c r="C293" s="1"/>
+    </row>
+    <row r="294" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B294" s="1"/>
+      <c r="C294" s="1"/>
+    </row>
+    <row r="295" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B295" s="1"/>
+      <c r="C295" s="1"/>
+    </row>
+    <row r="296" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B296" s="1"/>
+      <c r="C296" s="1"/>
+    </row>
+    <row r="297" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B297" s="1"/>
+      <c r="C297" s="1"/>
+    </row>
+    <row r="298" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B298" s="1"/>
+      <c r="C298" s="1"/>
+    </row>
+    <row r="299" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B299" s="1"/>
+      <c r="C299" s="1"/>
+    </row>
+    <row r="300" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B300" s="1"/>
+      <c r="C300" s="1"/>
+    </row>
+    <row r="301" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B301" s="1"/>
+      <c r="C301" s="1"/>
+    </row>
+    <row r="302" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B302" s="1"/>
+      <c r="C302" s="1"/>
+    </row>
+    <row r="303" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B303" s="1"/>
+      <c r="C303" s="1"/>
+    </row>
+    <row r="304" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B304" s="1"/>
+      <c r="C304" s="1"/>
+    </row>
+    <row r="305" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B305" s="1"/>
+      <c r="C305" s="1"/>
+    </row>
+    <row r="306" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B306" s="1"/>
+      <c r="C306" s="1"/>
+    </row>
+    <row r="307" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B307" s="1"/>
+      <c r="C307" s="1"/>
+    </row>
+    <row r="308" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B308" s="1"/>
+      <c r="C308" s="1"/>
+    </row>
+    <row r="309" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B309" s="1"/>
+      <c r="C309" s="1"/>
+    </row>
+    <row r="310" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B310" s="1"/>
+      <c r="C310" s="1"/>
+    </row>
+    <row r="311" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B311" s="1"/>
+      <c r="C311" s="1"/>
+    </row>
+    <row r="312" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B312" s="1"/>
+      <c r="C312" s="1"/>
+    </row>
+    <row r="313" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B313" s="1"/>
+      <c r="C313" s="1"/>
+    </row>
+    <row r="314" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B314" s="1"/>
+      <c r="C314" s="1"/>
+    </row>
+    <row r="315" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B315" s="1"/>
+      <c r="C315" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Updated log boek + delen van toDo list
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Mathijs.xlsx
+++ b/Logboeken/Logboek Mathijs.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="62">
   <si>
     <t>Datum</t>
   </si>
@@ -193,6 +193,18 @@
   </si>
   <si>
     <t>Begonnen met selectief laden van annotaties op de kaart</t>
+  </si>
+  <si>
+    <t>Meer bezig geweest met het selectief laden, methode is af maar zit nog een foutje in</t>
+  </si>
+  <si>
+    <t>Fout opgespoort, blijken nog meer fouten in de methode te staan</t>
+  </si>
+  <si>
+    <t>Deze fouten ook gefixed</t>
+  </si>
+  <si>
+    <t>Methode wordt te vaak aangeroepen, workaround verzinnen</t>
   </si>
 </sst>
 </file>
@@ -1198,107 +1210,144 @@
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="4"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
+      <c r="A55" s="3">
+        <v>41052</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
+      <c r="A56" s="3">
+        <v>41052</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
+      <c r="A57" s="3">
+        <v>41052</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
+      <c r="A58" s="3">
+        <v>41052</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="4"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="4"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="4"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="4"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="4"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="4"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="4"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="4"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
     </row>

</xml_diff>